<commit_message>
Update description,Mapping, déplacement des invariants 5f66202ed479bb7286b49ba09e288c70a36e347a
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-service-request-besoin.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-service-request-besoin.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T09:32:11+00:00</t>
+    <t>2026-06-24T08:54:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -525,9 +525,6 @@
 </t>
   </si>
   <si>
-    <t>idBesoin</t>
-  </si>
-  <si>
     <t>Request.identifier</t>
   </si>
   <si>
@@ -734,6 +731,9 @@
   </si>
   <si>
     <t>ServiceRequest.identifier:idBesoin</t>
+  </si>
+  <si>
+    <t>idBesoin</t>
   </si>
   <si>
     <t>Identifiant du besoin</t>
@@ -3534,30 +3534,30 @@
         <v>104</v>
       </c>
       <c r="AK12" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AL12" t="s" s="2">
         <v>163</v>
       </c>
-      <c r="AL12" t="s" s="2">
+      <c r="AM12" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="AM12" t="s" s="2">
+      <c r="AN12" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="AN12" t="s" s="2">
+      <c r="AO12" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="AO12" t="s" s="2">
+      <c r="AP12" t="s" s="2">
         <v>167</v>
-      </c>
-      <c r="AP12" t="s" s="2">
-        <v>168</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -3580,13 +3580,13 @@
         <v>82</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L13" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="L13" t="s" s="2">
+      <c r="M13" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="M13" t="s" s="2">
-        <v>172</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -3637,7 +3637,7 @@
         <v>82</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>80</v>
@@ -3661,7 +3661,7 @@
         <v>82</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO13" t="s" s="2">
         <v>82</v>
@@ -3672,10 +3672,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3701,10 +3701,10 @@
         <v>137</v>
       </c>
       <c r="L14" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="M14" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="N14" t="s" s="2">
         <v>154</v>
@@ -3748,7 +3748,7 @@
         <v>140</v>
       </c>
       <c r="AC14" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD14" t="s" s="2">
         <v>82</v>
@@ -3757,7 +3757,7 @@
         <v>141</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>80</v>
@@ -3781,7 +3781,7 @@
         <v>82</v>
       </c>
       <c r="AN14" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO14" t="s" s="2">
         <v>82</v>
@@ -3792,10 +3792,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3821,16 +3821,16 @@
         <v>112</v>
       </c>
       <c r="L15" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="M15" t="s" s="2">
         <v>181</v>
       </c>
-      <c r="M15" t="s" s="2">
+      <c r="N15" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="N15" t="s" s="2">
+      <c r="O15" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="O15" t="s" s="2">
-        <v>184</v>
       </c>
       <c r="P15" t="s" s="2">
         <v>82</v>
@@ -3855,31 +3855,31 @@
         <v>82</v>
       </c>
       <c r="X15" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="Y15" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="Y15" t="s" s="2">
+      <c r="Z15" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="Z15" t="s" s="2">
+      <c r="AA15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF15" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AA15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF15" t="s" s="2">
-        <v>188</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>80</v>
@@ -3903,7 +3903,7 @@
         <v>135</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AO15" t="s" s="2">
         <v>82</v>
@@ -3914,10 +3914,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3940,19 +3940,19 @@
         <v>93</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="L16" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="M16" t="s" s="2">
+      <c r="N16" t="s" s="2">
         <v>193</v>
       </c>
-      <c r="N16" t="s" s="2">
+      <c r="O16" t="s" s="2">
         <v>194</v>
-      </c>
-      <c r="O16" t="s" s="2">
-        <v>195</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>82</v>
@@ -3977,29 +3977,29 @@
         <v>82</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y16" s="2"/>
       <c r="Z16" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="AA16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF16" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="AA16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF16" t="s" s="2">
-        <v>197</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>80</v>
@@ -4020,10 +4020,10 @@
         <v>82</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AO16" t="s" s="2">
         <v>82</v>
@@ -4034,10 +4034,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -4063,16 +4063,16 @@
         <v>106</v>
       </c>
       <c r="L17" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="M17" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="N17" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="N17" t="s" s="2">
+      <c r="O17" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="O17" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>82</v>
@@ -4085,43 +4085,43 @@
         <v>82</v>
       </c>
       <c r="T17" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="U17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>204</v>
-      </c>
-      <c r="U17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>205</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>80</v>
@@ -4142,10 +4142,10 @@
         <v>82</v>
       </c>
       <c r="AM17" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="AN17" t="s" s="2">
         <v>206</v>
-      </c>
-      <c r="AN17" t="s" s="2">
-        <v>207</v>
       </c>
       <c r="AO17" t="s" s="2">
         <v>82</v>
@@ -4156,10 +4156,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -4182,16 +4182,16 @@
         <v>93</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L18" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="M18" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="M18" t="s" s="2">
+      <c r="N18" t="s" s="2">
         <v>210</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>211</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -4205,43 +4205,43 @@
         <v>82</v>
       </c>
       <c r="T18" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="U18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF18" t="s" s="2">
         <v>212</v>
-      </c>
-      <c r="U18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE18" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF18" t="s" s="2">
-        <v>213</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>80</v>
@@ -4262,10 +4262,10 @@
         <v>82</v>
       </c>
       <c r="AM18" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="AN18" t="s" s="2">
         <v>214</v>
-      </c>
-      <c r="AN18" t="s" s="2">
-        <v>215</v>
       </c>
       <c r="AO18" t="s" s="2">
         <v>82</v>
@@ -4276,10 +4276,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -4302,13 +4302,13 @@
         <v>93</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="L19" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="M19" t="s" s="2">
         <v>218</v>
-      </c>
-      <c r="M19" t="s" s="2">
-        <v>219</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -4359,7 +4359,7 @@
         <v>82</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>80</v>
@@ -4380,10 +4380,10 @@
         <v>82</v>
       </c>
       <c r="AM19" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="AN19" t="s" s="2">
         <v>221</v>
-      </c>
-      <c r="AN19" t="s" s="2">
-        <v>222</v>
       </c>
       <c r="AO19" t="s" s="2">
         <v>82</v>
@@ -4394,10 +4394,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4420,16 +4420,16 @@
         <v>93</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>223</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="M20" t="s" s="2">
         <v>225</v>
       </c>
-      <c r="M20" t="s" s="2">
+      <c r="N20" t="s" s="2">
         <v>226</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>227</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -4479,7 +4479,7 @@
         <v>82</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -4500,10 +4500,10 @@
         <v>82</v>
       </c>
       <c r="AM20" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="AN20" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="AN20" t="s" s="2">
-        <v>230</v>
       </c>
       <c r="AO20" t="s" s="2">
         <v>82</v>
@@ -4514,13 +4514,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B21" t="s" s="2">
         <v>157</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>163</v>
+        <v>231</v>
       </c>
       <c r="D21" t="s" s="2">
         <v>82</v>
@@ -4616,22 +4616,22 @@
         <v>104</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>82</v>
+        <v>231</v>
       </c>
       <c r="AL21" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="AM21" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="AM21" t="s" s="2">
+      <c r="AN21" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="AN21" t="s" s="2">
+      <c r="AO21" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="AO21" t="s" s="2">
+      <c r="AP21" t="s" s="2">
         <v>167</v>
-      </c>
-      <c r="AP21" t="s" s="2">
-        <v>168</v>
       </c>
     </row>
     <row r="22">
@@ -4639,7 +4639,7 @@
         <v>233</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4662,13 +4662,13 @@
         <v>82</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L22" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="L22" t="s" s="2">
+      <c r="M22" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>172</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -4719,7 +4719,7 @@
         <v>82</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -4743,7 +4743,7 @@
         <v>82</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>82</v>
@@ -4757,7 +4757,7 @@
         <v>234</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4783,10 +4783,10 @@
         <v>137</v>
       </c>
       <c r="L23" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="M23" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="N23" t="s" s="2">
         <v>154</v>
@@ -4830,7 +4830,7 @@
         <v>140</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>82</v>
@@ -4839,7 +4839,7 @@
         <v>141</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>80</v>
@@ -4863,7 +4863,7 @@
         <v>82</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO23" t="s" s="2">
         <v>82</v>
@@ -4877,7 +4877,7 @@
         <v>235</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4903,16 +4903,16 @@
         <v>112</v>
       </c>
       <c r="L24" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="M24" t="s" s="2">
         <v>181</v>
       </c>
-      <c r="M24" t="s" s="2">
+      <c r="N24" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="N24" t="s" s="2">
+      <c r="O24" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>184</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>82</v>
@@ -4937,31 +4937,31 @@
         <v>82</v>
       </c>
       <c r="X24" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="Y24" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="Y24" t="s" s="2">
+      <c r="Z24" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="Z24" t="s" s="2">
+      <c r="AA24" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB24" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD24" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE24" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF24" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AA24" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB24" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC24" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD24" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE24" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF24" t="s" s="2">
-        <v>188</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -4985,7 +4985,7 @@
         <v>135</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>82</v>
@@ -4999,7 +4999,7 @@
         <v>236</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -5022,19 +5022,19 @@
         <v>93</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="M25" t="s" s="2">
+      <c r="N25" t="s" s="2">
         <v>193</v>
       </c>
-      <c r="N25" t="s" s="2">
+      <c r="O25" t="s" s="2">
         <v>194</v>
-      </c>
-      <c r="O25" t="s" s="2">
-        <v>195</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>82</v>
@@ -5059,29 +5059,29 @@
         <v>82</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF25" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="AA25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE25" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF25" t="s" s="2">
-        <v>197</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
@@ -5102,10 +5102,10 @@
         <v>82</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AO25" t="s" s="2">
         <v>82</v>
@@ -5119,7 +5119,7 @@
         <v>238</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -5145,16 +5145,16 @@
         <v>106</v>
       </c>
       <c r="L26" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="M26" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="M26" t="s" s="2">
+      <c r="N26" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="N26" t="s" s="2">
+      <c r="O26" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="O26" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>82</v>
@@ -5167,43 +5167,43 @@
         <v>239</v>
       </c>
       <c r="T26" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF26" t="s" s="2">
         <v>204</v>
-      </c>
-      <c r="U26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE26" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF26" t="s" s="2">
-        <v>205</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -5224,10 +5224,10 @@
         <v>82</v>
       </c>
       <c r="AM26" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="AN26" t="s" s="2">
         <v>206</v>
-      </c>
-      <c r="AN26" t="s" s="2">
-        <v>207</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>82</v>
@@ -5241,7 +5241,7 @@
         <v>240</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -5264,16 +5264,16 @@
         <v>93</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="M27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>210</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>211</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -5287,43 +5287,43 @@
         <v>82</v>
       </c>
       <c r="T27" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>212</v>
-      </c>
-      <c r="U27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>213</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -5344,10 +5344,10 @@
         <v>82</v>
       </c>
       <c r="AM27" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="AN27" t="s" s="2">
         <v>214</v>
-      </c>
-      <c r="AN27" t="s" s="2">
-        <v>215</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>82</v>
@@ -5361,7 +5361,7 @@
         <v>242</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5384,13 +5384,13 @@
         <v>93</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>218</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>219</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -5441,7 +5441,7 @@
         <v>82</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -5462,10 +5462,10 @@
         <v>82</v>
       </c>
       <c r="AM28" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="AN28" t="s" s="2">
         <v>221</v>
-      </c>
-      <c r="AN28" t="s" s="2">
-        <v>222</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>82</v>
@@ -5479,7 +5479,7 @@
         <v>243</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5502,16 +5502,16 @@
         <v>93</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>223</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>225</v>
       </c>
-      <c r="M29" t="s" s="2">
+      <c r="N29" t="s" s="2">
         <v>226</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>227</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -5561,7 +5561,7 @@
         <v>82</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -5582,10 +5582,10 @@
         <v>82</v>
       </c>
       <c r="AM29" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="AN29" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="AN29" t="s" s="2">
-        <v>230</v>
       </c>
       <c r="AO29" t="s" s="2">
         <v>82</v>
@@ -6255,7 +6255,7 @@
         <v>82</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y35" t="s" s="2">
         <v>287</v>
@@ -6375,7 +6375,7 @@
         <v>82</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y36" t="s" s="2">
         <v>298</v>
@@ -6460,7 +6460,7 @@
         <v>93</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L37" t="s" s="2">
         <v>304</v>
@@ -6497,7 +6497,7 @@
         <v>82</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y37" s="2"/>
       <c r="Z37" t="s" s="2">
@@ -6615,7 +6615,7 @@
         <v>82</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y38" t="s" s="2">
         <v>316</v>
@@ -6824,7 +6824,7 @@
         <v>93</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L40" t="s" s="2">
         <v>333</v>
@@ -6944,13 +6944,13 @@
         <v>82</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>172</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -7001,7 +7001,7 @@
         <v>82</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -7025,7 +7025,7 @@
         <v>82</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO41" t="s" s="2">
         <v>82</v>
@@ -7065,10 +7065,10 @@
         <v>137</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="N42" t="s" s="2">
         <v>154</v>
@@ -7112,7 +7112,7 @@
         <v>140</v>
       </c>
       <c r="AC42" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD42" t="s" s="2">
         <v>82</v>
@@ -7121,7 +7121,7 @@
         <v>141</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -7145,7 +7145,7 @@
         <v>82</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>82</v>
@@ -7304,7 +7304,7 @@
         <v>93</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L44" t="s" s="2">
         <v>356</v>
@@ -7426,7 +7426,7 @@
         <v>93</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L45" t="s" s="2">
         <v>366</v>
@@ -7546,13 +7546,13 @@
         <v>82</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>172</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7603,7 +7603,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -7627,7 +7627,7 @@
         <v>82</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO46" t="s" s="2">
         <v>82</v>
@@ -7667,10 +7667,10 @@
         <v>137</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="N47" t="s" s="2">
         <v>154</v>
@@ -7714,7 +7714,7 @@
         <v>140</v>
       </c>
       <c r="AC47" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD47" t="s" s="2">
         <v>82</v>
@@ -7723,7 +7723,7 @@
         <v>141</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7747,7 +7747,7 @@
         <v>82</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO47" t="s" s="2">
         <v>82</v>
@@ -7906,7 +7906,7 @@
         <v>93</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L49" t="s" s="2">
         <v>356</v>
@@ -8858,7 +8858,7 @@
         <v>93</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L57" t="s" s="2">
         <v>444</v>
@@ -9098,7 +9098,7 @@
         <v>93</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L59" t="s" s="2">
         <v>463</v>
@@ -9334,7 +9334,7 @@
         <v>93</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L61" t="s" s="2">
         <v>473</v>
@@ -9932,7 +9932,7 @@
         <v>93</v>
       </c>
       <c r="K66" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L66" t="s" s="2">
         <v>515</v>
@@ -10172,13 +10172,13 @@
         <v>82</v>
       </c>
       <c r="K68" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L68" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="L68" t="s" s="2">
+      <c r="M68" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="M68" t="s" s="2">
-        <v>172</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -10229,7 +10229,7 @@
         <v>82</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>80</v>
@@ -10253,7 +10253,7 @@
         <v>82</v>
       </c>
       <c r="AN68" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO68" t="s" s="2">
         <v>82</v>
@@ -10293,10 +10293,10 @@
         <v>137</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="N69" t="s" s="2">
         <v>154</v>
@@ -10340,7 +10340,7 @@
         <v>140</v>
       </c>
       <c r="AC69" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD69" t="s" s="2">
         <v>82</v>
@@ -10349,7 +10349,7 @@
         <v>141</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>80</v>
@@ -10373,7 +10373,7 @@
         <v>82</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO69" t="s" s="2">
         <v>82</v>
@@ -10766,7 +10766,7 @@
         <v>93</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L73" t="s" s="2">
         <v>551</v>

</xml_diff>